<commit_message>
fix: supprime la contrainte note 0..1 ajoutée par Document Core d30870c74fe8ac8d1558eaa89ece11317577dead
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-statement.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication-statement.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-16T16:12:39+00:00</t>
+    <t>2026-07-20T14:23:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -4619,7 +4619,7 @@
         <v>79</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>78</v>

</xml_diff>